<commit_message>
Normalize bSYM to Dx across FAERS BERT and LLaMA evaluations, update Figure 5 and manuscript
</commit_message>
<xml_diff>
--- a/publication/results/bert_runs_FAERS_LOO/metrics.xlsx
+++ b/publication/results/bert_runs_FAERS_LOO/metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="All_Runs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fold_Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Per_Category" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Category_Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Runs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fold_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per_Category" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category_Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,10 +576,10 @@
         <v>5856</v>
       </c>
       <c r="F3" t="n">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="G3" t="n">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="H3" t="n">
         <v>1908</v>
@@ -630,10 +630,10 @@
         <v>6280</v>
       </c>
       <c r="F4" t="n">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="G4" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="H4" t="n">
         <v>1962</v>
@@ -681,16 +681,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6085</v>
+        <v>6086</v>
       </c>
       <c r="F5" t="n">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="G5" t="n">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="H5" t="n">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="I5" t="n">
         <v>3195</v>
@@ -699,22 +699,22 @@
         <v>1451</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5441</v>
+        <v>0.5442</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6446</v>
+        <v>0.6447000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5901</v>
+        <v>0.5901999999999999</v>
       </c>
       <c r="N5" t="n">
         <v>0.8008</v>
       </c>
       <c r="O5" t="n">
-        <v>0.7454</v>
+        <v>0.7455000000000001</v>
       </c>
       <c r="P5" t="n">
-        <v>0.7721</v>
+        <v>0.7722</v>
       </c>
     </row>
     <row r="6">
@@ -1386,10 +1386,10 @@
         <v>7574</v>
       </c>
       <c r="F18" t="n">
-        <v>2122</v>
+        <v>2123</v>
       </c>
       <c r="G18" t="n">
-        <v>1547</v>
+        <v>1546</v>
       </c>
       <c r="H18" t="n">
         <v>3669</v>
@@ -1440,10 +1440,10 @@
         <v>7680</v>
       </c>
       <c r="F19" t="n">
-        <v>1870</v>
+        <v>1871</v>
       </c>
       <c r="G19" t="n">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="H19" t="n">
         <v>3562</v>
@@ -1494,10 +1494,10 @@
         <v>7465</v>
       </c>
       <c r="F20" t="n">
-        <v>2031</v>
+        <v>2033</v>
       </c>
       <c r="G20" t="n">
-        <v>1406</v>
+        <v>1404</v>
       </c>
       <c r="H20" t="n">
         <v>3437</v>
@@ -1677,16 +1677,16 @@
         <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>30318</v>
+        <v>30319</v>
       </c>
       <c r="E2" t="n">
-        <v>4713</v>
+        <v>4717</v>
       </c>
       <c r="F2" t="n">
-        <v>4481</v>
+        <v>4476</v>
       </c>
       <c r="G2" t="n">
-        <v>9194</v>
+        <v>9193</v>
       </c>
       <c r="H2" t="n">
         <v>14319</v>
@@ -1698,7 +1698,7 @@
         <v>0.6002</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0114</v>
+        <v>0.0113</v>
       </c>
       <c r="L2" t="n">
         <v>0.7733</v>
@@ -1815,10 +1815,10 @@
         <v>37786</v>
       </c>
       <c r="E5" t="n">
-        <v>10153</v>
+        <v>10157</v>
       </c>
       <c r="F5" t="n">
-        <v>7984</v>
+        <v>7980</v>
       </c>
       <c r="G5" t="n">
         <v>18137</v>
@@ -2769,10 +2769,10 @@
         <v>367</v>
       </c>
       <c r="F17" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G17" t="n">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="H17" t="n">
         <v>594</v>
@@ -3957,10 +3957,10 @@
         <v>536</v>
       </c>
       <c r="F39" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G39" t="n">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H39" t="n">
         <v>653</v>
@@ -4548,16 +4548,16 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F50" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G50" t="n">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="H50" t="n">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="I50" t="n">
         <v>405</v>
@@ -4566,22 +4566,22 @@
         <v>239</v>
       </c>
       <c r="K50" t="n">
-        <v>0.3061</v>
+        <v>0.3067</v>
       </c>
       <c r="L50" t="n">
-        <v>0.3437</v>
+        <v>0.3444</v>
       </c>
       <c r="M50" t="n">
-        <v>0.3238</v>
+        <v>0.3245</v>
       </c>
       <c r="N50" t="n">
-        <v>0.6496</v>
+        <v>0.65</v>
       </c>
       <c r="O50" t="n">
-        <v>0.5833</v>
+        <v>0.5837</v>
       </c>
       <c r="P50" t="n">
-        <v>0.6147</v>
+        <v>0.6151</v>
       </c>
     </row>
     <row r="51">
@@ -11679,10 +11679,10 @@
         <v>515</v>
       </c>
       <c r="F182" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G182" t="n">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="H182" t="n">
         <v>950</v>
@@ -12867,10 +12867,10 @@
         <v>563</v>
       </c>
       <c r="F204" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G204" t="n">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H204" t="n">
         <v>890</v>
@@ -13461,10 +13461,10 @@
         <v>503</v>
       </c>
       <c r="F215" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G215" t="n">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="H215" t="n">
         <v>883</v>
@@ -14064,16 +14064,16 @@
         <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>6093</v>
+        <v>6094</v>
       </c>
       <c r="D6" t="n">
-        <v>1447</v>
+        <v>1455</v>
       </c>
       <c r="E6" t="n">
-        <v>7586</v>
+        <v>7577</v>
       </c>
       <c r="F6" t="n">
-        <v>9033</v>
+        <v>9032</v>
       </c>
       <c r="G6" t="n">
         <v>4500</v>
@@ -14082,16 +14082,16 @@
         <v>3027</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3445</v>
+        <v>0.3446</v>
       </c>
       <c r="J6" t="n">
         <v>0.0515</v>
       </c>
       <c r="K6" t="n">
-        <v>0.628</v>
+        <v>0.6281</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0336</v>
+        <v>0.0335</v>
       </c>
     </row>
     <row r="7">

</xml_diff>